<commit_message>
Show fixed ICD columns C-K with editable newline choices from M
</commit_message>
<xml_diff>
--- a/prototype/examples/example-icd.xlsx
+++ b/prototype/examples/example-icd.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,7 +488,47 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>데이터 상세 값</t>
+          <t>고정 설명</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>가상 자료형</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>가상 크기</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>가상 최소</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>가상 최대</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>가상 초기</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>고정 비고</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>미사용</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>사용자 선택값</t>
         </is>
       </c>
     </row>
@@ -513,8 +553,41 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OFF ON	AUTO
-HOLD</t>
+          <t>고정 0 1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>uint8 예시</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>255</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>원본 유지</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>사용하지 않는 L열</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>정지 상태
+수동 운용
+자동 운용</t>
         </is>
       </c>
     </row>
@@ -529,7 +602,41 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1 2 3</t>
+          <t>고정 0 1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>uint8 예시</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>255</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>원본 유지</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>사용하지 않는 L열</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1
+2
+3</t>
         </is>
       </c>
     </row>
@@ -552,6 +659,38 @@
           <t>비고</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>고정 0 1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>uint8 예시</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>255</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>원본 유지</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>사용하지 않는 L열</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -574,7 +713,41 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>A B A</t>
+          <t>고정 0 1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>uint8 예시</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>255</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>원본 유지</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>사용하지 않는 L열</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>A
+B
+A</t>
         </is>
       </c>
     </row>
@@ -593,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,7 +792,47 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>데이터 상세 값</t>
+          <t>고정 설명</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>가상 자료형</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>가상 크기</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>가상 최소</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>가상 최대</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>가상 초기</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>고정 비고</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>미사용</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>사용자 선택값</t>
         </is>
       </c>
     </row>
@@ -644,7 +857,41 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>LOW MEDIUM HIGH</t>
+          <t>고정 0 1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>uint8 예시</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>255</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>원본 유지</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>사용하지 않는 L열</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>LOW
+MEDIUM
+HIGH</t>
         </is>
       </c>
     </row>
@@ -655,6 +902,38 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>설명</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>고정 0 1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>uint8 예시</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>255</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>원본 유지</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>사용하지 않는 L열</t>
         </is>
       </c>
     </row>

</xml_diff>